<commit_message>
Keep Hyperdrive off dual-court ref duties
Hyperdrive only has 7 players, so they cannot cover both courts. Restructure
to 4 dual-court rounds (other teams each bye/dual-ref once) plus 2 single-court
rounds that Hyperdrive refs alone. Still 2 home / 2 away / 2 refs for every team.

Co-authored-by: Jess Sartin <jdoherty513@gmail.com>
</commit_message>
<xml_diff>
--- a/public/league_schedules/Five Team Round Robin.xlsx
+++ b/public/league_schedules/Five Team Round Robin.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,30 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Five Team Round Robin</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cannot dual-ref</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hyperdrive has fewer than 8 players and refs one court at a time only</t>
         </is>
       </c>
     </row>
@@ -803,7 +827,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>'Week 1'!B23</f>
+        <f>'Week 1'!B27</f>
         <v/>
       </c>
       <c r="C17">
@@ -811,7 +835,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>'Week 1'!C23</f>
+        <f>'Week 1'!C27</f>
         <v/>
       </c>
     </row>
@@ -822,7 +846,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>'Week 1'!B24</f>
+        <f>'Week 1'!B28</f>
         <v/>
       </c>
       <c r="C18">
@@ -830,7 +854,7 @@
         <v/>
       </c>
       <c r="E18">
-        <f>'Week 1'!C24</f>
+        <f>'Week 1'!C28</f>
         <v/>
       </c>
     </row>
@@ -841,7 +865,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>'Week 1'!B25</f>
+        <f>'Week 1'!B29</f>
         <v/>
       </c>
       <c r="C19">
@@ -849,7 +873,7 @@
         <v/>
       </c>
       <c r="E19">
-        <f>'Week 1'!C25</f>
+        <f>'Week 1'!C29</f>
         <v/>
       </c>
     </row>
@@ -860,7 +884,7 @@
         </is>
       </c>
       <c r="B20">
-        <f>'Week 1'!B26</f>
+        <f>'Week 1'!B30</f>
         <v/>
       </c>
       <c r="C20">
@@ -868,7 +892,7 @@
         <v/>
       </c>
       <c r="E20">
-        <f>'Week 1'!C26</f>
+        <f>'Week 1'!C30</f>
         <v/>
       </c>
     </row>
@@ -879,7 +903,7 @@
         </is>
       </c>
       <c r="B21">
-        <f>'Week 1'!B27</f>
+        <f>'Week 1'!B31</f>
         <v/>
       </c>
       <c r="C21">
@@ -887,7 +911,7 @@
         <v/>
       </c>
       <c r="E21">
-        <f>'Week 1'!C27</f>
+        <f>'Week 1'!C31</f>
         <v/>
       </c>
     </row>
@@ -902,7 +926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -925,22 +949,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>Full Throttle</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>High Octane</t>
         </is>
       </c>
     </row>
@@ -964,34 +988,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Carbon Fiber</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Full Throttle</t>
+          <t>(no game — single court)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Refs: High Octane</t>
+          <t>Refs: Hyperdrive</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Refs: High Octane</t>
+          <t>Hyperdrive — Court 1 only (cannot cover both courts)</t>
         </is>
       </c>
     </row>
@@ -1003,22 +1022,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Full Throttle</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>Carbon Fiber</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>High Octane</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Full Throttle</t>
         </is>
       </c>
     </row>
@@ -1042,34 +1061,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>High Octane</t>
+          <t>Hyperdrive</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Full Throttle</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>Carbon Fiber</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Refs: Full Throttle</t>
+          <t>Refs: High Octane</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Refs: Full Throttle</t>
+          <t>Refs: High Octane</t>
         </is>
       </c>
     </row>
@@ -1086,17 +1105,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
+          <t>Velocity Syndicate</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>High Octane</t>
+          <t>(no game — single court)</t>
         </is>
       </c>
     </row>
@@ -1108,75 +1122,82 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Refs: Hyperdrive</t>
+          <t>Hyperdrive — Court 1 only (cannot cover both courts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Game 06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>High Octane</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Balance check (home / away / refs)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Refs</t>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Refs: Full Throttle</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Refs: Full Throttle</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" t="n">
-        <v>2</v>
+          <t>Balance check (home / away / refs)</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>2</v>
-      </c>
-      <c r="C16" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" t="n">
-        <v>2</v>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Refs</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Hyperdrive</t>
+          <t>Carbon Fiber</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1192,7 +1213,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>High Octane</t>
+          <t>Velocity Syndicate</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1208,7 +1229,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Full Throttle</t>
+          <t>Hyperdrive</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1218,104 +1239,143 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Team Wins/Losses This Week</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Team Name</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Wins</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
+          <t>Full Throttle</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>SUMIFS(C:C,B:B,"Carbon Fiber*")+SUMIFS(E:E,D:D,"Carbon Fiber*")+SUMIFS(H:H,G:G,"Carbon Fiber*")+SUMIFS(J:J,I:I,"Carbon Fiber*")</f>
-        <v/>
-      </c>
-      <c r="C23">
-        <f>SUMIFS(E:E,B:B,"Carbon Fiber*")+SUMIFS(C:C,D:D,"Carbon Fiber*")+SUMIFS(J:J,G:G,"Carbon Fiber*")+SUMIFS(H:H,I:I,"Carbon Fiber*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="B24">
-        <f>SUMIFS(C:C,B:B,"Velocity Syndicate*")+SUMIFS(E:E,D:D,"Velocity Syndicate*")+SUMIFS(H:H,G:G,"Velocity Syndicate*")+SUMIFS(J:J,I:I,"Velocity Syndicate*")</f>
-        <v/>
-      </c>
-      <c r="C24">
-        <f>SUMIFS(E:E,B:B,"Velocity Syndicate*")+SUMIFS(C:C,D:D,"Velocity Syndicate*")+SUMIFS(J:J,G:G,"Velocity Syndicate*")+SUMIFS(H:H,I:I,"Velocity Syndicate*")</f>
-        <v/>
+          <t>Note: Hyperdrive cannot ref both courts (7 players); they ref Court 1 only in the two single-court rounds.</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>SUMIFS(C:C,B:B,"Hyperdrive")+SUMIFS(E:E,D:D,"Hyperdrive")+SUMIFS(H:H,G:G,"Hyperdrive")+SUMIFS(J:J,I:I,"Hyperdrive")</f>
-        <v/>
-      </c>
-      <c r="C25">
-        <f>SUMIFS(E:E,B:B,"Hyperdrive")+SUMIFS(C:C,D:D,"Hyperdrive")+SUMIFS(J:J,G:G,"Hyperdrive")+SUMIFS(H:H,I:I,"Hyperdrive")</f>
-        <v/>
+          <t>Team Wins/Losses This Week</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>High Octane</t>
-        </is>
-      </c>
-      <c r="B26">
-        <f>SUMIFS(C:C,B:B,"High Octane*")+SUMIFS(E:E,D:D,"High Octane*")+SUMIFS(H:H,G:G,"High Octane*")+SUMIFS(J:J,I:I,"High Octane*")</f>
-        <v/>
-      </c>
-      <c r="C26">
-        <f>SUMIFS(E:E,B:B,"High Octane*")+SUMIFS(C:C,D:D,"High Octane*")+SUMIFS(J:J,G:G,"High Octane*")+SUMIFS(H:H,I:I,"High Octane*")</f>
-        <v/>
+          <t>Team Name</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>SUMIFS(C:C,B:B,"Carbon Fiber*")+SUMIFS(E:E,D:D,"Carbon Fiber*")+SUMIFS(H:H,G:G,"Carbon Fiber*")+SUMIFS(J:J,I:I,"Carbon Fiber*")</f>
+        <v/>
+      </c>
+      <c r="C27">
+        <f>SUMIFS(E:E,B:B,"Carbon Fiber*")+SUMIFS(C:C,D:D,"Carbon Fiber*")+SUMIFS(J:J,G:G,"Carbon Fiber*")+SUMIFS(H:H,I:I,"Carbon Fiber*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>SUMIFS(C:C,B:B,"Velocity Syndicate*")+SUMIFS(E:E,D:D,"Velocity Syndicate*")+SUMIFS(H:H,G:G,"Velocity Syndicate*")+SUMIFS(J:J,I:I,"Velocity Syndicate*")</f>
+        <v/>
+      </c>
+      <c r="C28">
+        <f>SUMIFS(E:E,B:B,"Velocity Syndicate*")+SUMIFS(C:C,D:D,"Velocity Syndicate*")+SUMIFS(J:J,G:G,"Velocity Syndicate*")+SUMIFS(H:H,I:I,"Velocity Syndicate*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>SUMIFS(C:C,B:B,"Hyperdrive")+SUMIFS(E:E,D:D,"Hyperdrive")+SUMIFS(H:H,G:G,"Hyperdrive")+SUMIFS(J:J,I:I,"Hyperdrive")</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>SUMIFS(E:E,B:B,"Hyperdrive")+SUMIFS(C:C,D:D,"Hyperdrive")+SUMIFS(J:J,G:G,"Hyperdrive")+SUMIFS(H:H,I:I,"Hyperdrive")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>SUMIFS(C:C,B:B,"High Octane*")+SUMIFS(E:E,D:D,"High Octane*")+SUMIFS(H:H,G:G,"High Octane*")+SUMIFS(J:J,I:I,"High Octane*")</f>
+        <v/>
+      </c>
+      <c r="C30">
+        <f>SUMIFS(E:E,B:B,"High Octane*")+SUMIFS(C:C,D:D,"High Octane*")+SUMIFS(J:J,G:G,"High Octane*")+SUMIFS(H:H,I:I,"High Octane*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Full Throttle</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B31">
         <f>SUMIFS(C:C,B:B,"Full Throttle*")+SUMIFS(E:E,D:D,"Full Throttle*")+SUMIFS(H:H,G:G,"Full Throttle*")+SUMIFS(J:J,I:I,"Full Throttle*")</f>
         <v/>
       </c>
-      <c r="C27">
+      <c r="C31">
         <f>SUMIFS(E:E,B:B,"Full Throttle*")+SUMIFS(C:C,D:D,"Full Throttle*")+SUMIFS(J:J,G:G,"Full Throttle*")+SUMIFS(H:H,I:I,"Full Throttle*")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Revert to original 5-round dual-court round-robin
Restore the first schedule: five dual-court rounds, bye team refs both
courts, every team 2 home / 2 away / 2 refs (including Hyperdrive).

Co-authored-by: Jess Sartin <jdoherty513@gmail.com>
</commit_message>
<xml_diff>
--- a/public/league_schedules/Five Team Round Robin.xlsx
+++ b/public/league_schedules/Five Team Round Robin.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,30 +472,6 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Five Team Round Robin</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Cannot dual-ref</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hyperdrive has fewer than 8 players and refs one court at a time only</t>
         </is>
       </c>
     </row>
@@ -827,7 +803,7 @@
         </is>
       </c>
       <c r="B17">
-        <f>'Week 1'!B27</f>
+        <f>'Week 1'!B23</f>
         <v/>
       </c>
       <c r="C17">
@@ -835,7 +811,7 @@
         <v/>
       </c>
       <c r="E17">
-        <f>'Week 1'!C27</f>
+        <f>'Week 1'!C23</f>
         <v/>
       </c>
     </row>
@@ -846,7 +822,7 @@
         </is>
       </c>
       <c r="B18">
-        <f>'Week 1'!B28</f>
+        <f>'Week 1'!B24</f>
         <v/>
       </c>
       <c r="C18">
@@ -854,7 +830,7 @@
         <v/>
       </c>
       <c r="E18">
-        <f>'Week 1'!C28</f>
+        <f>'Week 1'!C24</f>
         <v/>
       </c>
     </row>
@@ -865,7 +841,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>'Week 1'!B29</f>
+        <f>'Week 1'!B25</f>
         <v/>
       </c>
       <c r="C19">
@@ -873,7 +849,7 @@
         <v/>
       </c>
       <c r="E19">
-        <f>'Week 1'!C29</f>
+        <f>'Week 1'!C25</f>
         <v/>
       </c>
     </row>
@@ -884,7 +860,7 @@
         </is>
       </c>
       <c r="B20">
-        <f>'Week 1'!B30</f>
+        <f>'Week 1'!B26</f>
         <v/>
       </c>
       <c r="C20">
@@ -892,7 +868,7 @@
         <v/>
       </c>
       <c r="E20">
-        <f>'Week 1'!C30</f>
+        <f>'Week 1'!C26</f>
         <v/>
       </c>
     </row>
@@ -903,7 +879,7 @@
         </is>
       </c>
       <c r="B21">
-        <f>'Week 1'!B31</f>
+        <f>'Week 1'!B27</f>
         <v/>
       </c>
       <c r="C21">
@@ -911,7 +887,7 @@
         <v/>
       </c>
       <c r="E21">
-        <f>'Week 1'!C31</f>
+        <f>'Week 1'!C27</f>
         <v/>
       </c>
     </row>
@@ -926,7 +902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -949,22 +925,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Full Throttle</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Velocity Syndicate</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Hyperdrive</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>High Octane</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Full Throttle</t>
         </is>
       </c>
     </row>
@@ -988,29 +964,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>High Octane</t>
+          <t>Carbon Fiber</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
+          <t>Velocity Syndicate</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>(no game — single court)</t>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Full Throttle</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Refs: Hyperdrive</t>
+          <t>Refs: High Octane</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Hyperdrive — Court 1 only (cannot cover both courts)</t>
+          <t>Refs: High Octane</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1003,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Hyperdrive</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>High Octane</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Full Throttle</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Carbon Fiber</t>
         </is>
       </c>
     </row>
@@ -1061,34 +1042,34 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Full Throttle</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Carbon Fiber</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Refs: High Octane</t>
+          <t>Refs: Full Throttle</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Refs: High Octane</t>
+          <t>Refs: Full Throttle</t>
         </is>
       </c>
     </row>
@@ -1105,12 +1086,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>Velocity Syndicate</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>(no game — single court)</t>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>High Octane</t>
         </is>
       </c>
     </row>
@@ -1122,82 +1108,75 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Hyperdrive — Court 1 only (cannot cover both courts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Game 06</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Carbon Fiber</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>High Octane</t>
+          <t>Refs: Hyperdrive</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Refs: Full Throttle</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Refs: Full Throttle</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Balance check (home / away / refs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Refs</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Balance check (home / away / refs)</t>
-        </is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Refs</t>
-        </is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
+          <t>Hyperdrive</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1213,7 +1192,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Velocity Syndicate</t>
+          <t>High Octane</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1229,7 +1208,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Hyperdrive</t>
+          <t>Full Throttle</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1239,143 +1218,104 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>High Octane</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Full Throttle</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>2</v>
+          <t>Team Wins/Losses This Week</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Team Name</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Note: Hyperdrive cannot ref both courts (7 players); they ref Court 1 only in the two single-court rounds.</t>
-        </is>
+          <t>Carbon Fiber</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>SUMIFS(C:C,B:B,"Carbon Fiber*")+SUMIFS(E:E,D:D,"Carbon Fiber*")+SUMIFS(H:H,G:G,"Carbon Fiber*")+SUMIFS(J:J,I:I,"Carbon Fiber*")</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>SUMIFS(E:E,B:B,"Carbon Fiber*")+SUMIFS(C:C,D:D,"Carbon Fiber*")+SUMIFS(J:J,G:G,"Carbon Fiber*")+SUMIFS(H:H,I:I,"Carbon Fiber*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Velocity Syndicate</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>SUMIFS(C:C,B:B,"Velocity Syndicate*")+SUMIFS(E:E,D:D,"Velocity Syndicate*")+SUMIFS(H:H,G:G,"Velocity Syndicate*")+SUMIFS(J:J,I:I,"Velocity Syndicate*")</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>SUMIFS(E:E,B:B,"Velocity Syndicate*")+SUMIFS(C:C,D:D,"Velocity Syndicate*")+SUMIFS(J:J,G:G,"Velocity Syndicate*")+SUMIFS(H:H,I:I,"Velocity Syndicate*")</f>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Team Wins/Losses This Week</t>
-        </is>
+          <t>Hyperdrive</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>SUMIFS(C:C,B:B,"Hyperdrive")+SUMIFS(E:E,D:D,"Hyperdrive")+SUMIFS(H:H,G:G,"Hyperdrive")+SUMIFS(J:J,I:I,"Hyperdrive")</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>SUMIFS(E:E,B:B,"Hyperdrive")+SUMIFS(C:C,D:D,"Hyperdrive")+SUMIFS(J:J,G:G,"Hyperdrive")+SUMIFS(H:H,I:I,"Hyperdrive")</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Team Name</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Wins</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
+          <t>High Octane</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>SUMIFS(C:C,B:B,"High Octane*")+SUMIFS(E:E,D:D,"High Octane*")+SUMIFS(H:H,G:G,"High Octane*")+SUMIFS(J:J,I:I,"High Octane*")</f>
+        <v/>
+      </c>
+      <c r="C26">
+        <f>SUMIFS(E:E,B:B,"High Octane*")+SUMIFS(C:C,D:D,"High Octane*")+SUMIFS(J:J,G:G,"High Octane*")+SUMIFS(H:H,I:I,"High Octane*")</f>
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Carbon Fiber</t>
+          <t>Full Throttle</t>
         </is>
       </c>
       <c r="B27">
-        <f>SUMIFS(C:C,B:B,"Carbon Fiber*")+SUMIFS(E:E,D:D,"Carbon Fiber*")+SUMIFS(H:H,G:G,"Carbon Fiber*")+SUMIFS(J:J,I:I,"Carbon Fiber*")</f>
+        <f>SUMIFS(C:C,B:B,"Full Throttle*")+SUMIFS(E:E,D:D,"Full Throttle*")+SUMIFS(H:H,G:G,"Full Throttle*")+SUMIFS(J:J,I:I,"Full Throttle*")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>SUMIFS(E:E,B:B,"Carbon Fiber*")+SUMIFS(C:C,D:D,"Carbon Fiber*")+SUMIFS(J:J,G:G,"Carbon Fiber*")+SUMIFS(H:H,I:I,"Carbon Fiber*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Velocity Syndicate</t>
-        </is>
-      </c>
-      <c r="B28">
-        <f>SUMIFS(C:C,B:B,"Velocity Syndicate*")+SUMIFS(E:E,D:D,"Velocity Syndicate*")+SUMIFS(H:H,G:G,"Velocity Syndicate*")+SUMIFS(J:J,I:I,"Velocity Syndicate*")</f>
-        <v/>
-      </c>
-      <c r="C28">
-        <f>SUMIFS(E:E,B:B,"Velocity Syndicate*")+SUMIFS(C:C,D:D,"Velocity Syndicate*")+SUMIFS(J:J,G:G,"Velocity Syndicate*")+SUMIFS(H:H,I:I,"Velocity Syndicate*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Hyperdrive</t>
-        </is>
-      </c>
-      <c r="B29">
-        <f>SUMIFS(C:C,B:B,"Hyperdrive")+SUMIFS(E:E,D:D,"Hyperdrive")+SUMIFS(H:H,G:G,"Hyperdrive")+SUMIFS(J:J,I:I,"Hyperdrive")</f>
-        <v/>
-      </c>
-      <c r="C29">
-        <f>SUMIFS(E:E,B:B,"Hyperdrive")+SUMIFS(C:C,D:D,"Hyperdrive")+SUMIFS(J:J,G:G,"Hyperdrive")+SUMIFS(H:H,I:I,"Hyperdrive")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>High Octane</t>
-        </is>
-      </c>
-      <c r="B30">
-        <f>SUMIFS(C:C,B:B,"High Octane*")+SUMIFS(E:E,D:D,"High Octane*")+SUMIFS(H:H,G:G,"High Octane*")+SUMIFS(J:J,I:I,"High Octane*")</f>
-        <v/>
-      </c>
-      <c r="C30">
-        <f>SUMIFS(E:E,B:B,"High Octane*")+SUMIFS(C:C,D:D,"High Octane*")+SUMIFS(J:J,G:G,"High Octane*")+SUMIFS(H:H,I:I,"High Octane*")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Full Throttle</t>
-        </is>
-      </c>
-      <c r="B31">
-        <f>SUMIFS(C:C,B:B,"Full Throttle*")+SUMIFS(E:E,D:D,"Full Throttle*")+SUMIFS(H:H,G:G,"Full Throttle*")+SUMIFS(J:J,I:I,"Full Throttle*")</f>
-        <v/>
-      </c>
-      <c r="C31">
         <f>SUMIFS(E:E,B:B,"Full Throttle*")+SUMIFS(C:C,D:D,"Full Throttle*")+SUMIFS(J:J,G:G,"Full Throttle*")+SUMIFS(H:H,I:I,"Full Throttle*")</f>
         <v/>
       </c>

</xml_diff>